<commit_message>
Differentiate CellSens (login) and Preciv (dashboard) test modules
</commit_message>
<xml_diff>
--- a/test_suites/CellSens/Regression Testing/login_test_cases.xlsx
+++ b/test_suites/CellSens/Regression Testing/login_test_cases.xlsx
@@ -169,20 +169,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -441,73 +437,73 @@
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>